<commit_message>
updates after reruns with eSMR bugfix
</commit_message>
<xml_diff>
--- a/Plotting/Latex/filtered_data.xlsx
+++ b/Plotting/Latex/filtered_data.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,7 +598,7 @@
         <v>497</v>
       </c>
       <c r="I4" t="n">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -661,7 +661,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -859,7 +859,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>481</v>
+        <v>375</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -1055,13 +1055,17 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>1078</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1078</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1124,11 +1128,15 @@
       <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
-        <v>87</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1164,22 +1172,22 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>784</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>617</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1242,15 +1250,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="L14" t="n">
+        <v>784</v>
+      </c>
+      <c r="M14" t="n">
+        <v>784</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1286,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -1295,13 +1299,13 @@
         <v>1277</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>198</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>1026</v>
+        <v>895</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -1364,15 +1368,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="L16" t="n">
+        <v>198</v>
+      </c>
+      <c r="M16" t="n">
+        <v>198</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>262</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1559,67 +1559,53 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="L20" t="n">
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Methanol synthesis from syngas existing</t>
+          <t>Direct methanol synthesis from \ce{CO2}</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>t syngas/h</t>
+          <t>t \ce{CO2}/h</t>
         </is>
       </c>
     </row>
@@ -1627,21 +1613,17 @@
       <c r="A21" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B21" t="n">
+        <v>497</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>486</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>377</v>
+      </c>
+      <c r="E21" t="n">
+        <v>497</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1649,36 +1631,32 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H21" t="n">
+        <v>0</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>159</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Direct methanol synthesis from \ce{CO2}</t>
+          <t>\acs{MTO}</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>t \ce{CO2}/h</t>
+          <t>t methanol/h</t>
         </is>
       </c>
     </row>
@@ -1686,45 +1664,63 @@
       <c r="A22" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
         <v>497</v>
       </c>
-      <c r="C22" t="n">
-        <v>486</v>
-      </c>
-      <c r="D22" t="n">
-        <v>377</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="G22" t="n">
         <v>497</v>
       </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>16</v>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>\acs{MTO}</t>
+          <t>\acs{MTO} existing</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1737,68 +1733,50 @@
       <c r="A23" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>497</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>497</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>\acs{MTO} existing</t>
+          <t>\acs{EDH}</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>t methanol/h</t>
+          <t>t ethanol/h</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1785,7 @@
         <v>20</v>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -1816,7 +1794,7 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1837,19 +1815,19 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>\acs{EDH}</t>
+          <t>\acs{PDH}</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>t ethanol/h</t>
+          <t>t propane/h</t>
         </is>
       </c>
     </row>
@@ -1857,45 +1835,63 @@
       <c r="A25" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>64</v>
       </c>
-      <c r="C25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="G25" t="n">
         <v>64</v>
       </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>139</v>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M25" t="n">
-        <v>62</v>
+        <v>149</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>\acs{PDH}</t>
+          <t>\acs{PDH} existing</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -1908,68 +1904,50 @@
       <c r="A26" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B26" t="n">
+        <v>338</v>
+      </c>
+      <c r="C26" t="n">
+        <v>331</v>
+      </c>
+      <c r="D26" t="n">
+        <v>257</v>
+      </c>
+      <c r="E26" t="n">
+        <v>338</v>
       </c>
       <c r="F26" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>64</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>25</v>
       </c>
       <c r="M26" t="n">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>\acs{PDH} existing</t>
+          <t>\acs{MPW}-to-methanol</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>t propane/h</t>
+          <t>t MPW/h</t>
         </is>
       </c>
     </row>
@@ -1978,16 +1956,16 @@
         <v>23</v>
       </c>
       <c r="B27" t="n">
-        <v>338</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>331</v>
+        <v>34</v>
       </c>
       <c r="D27" t="n">
-        <v>257</v>
+        <v>58</v>
       </c>
       <c r="E27" t="n">
-        <v>338</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2008,19 +1986,19 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>\acs{MPW}-to-methanol</t>
+          <t>\acs{MPW}-to-methanol with \acs{CC}</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>t MPW/h</t>
+          <t>\% captured</t>
         </is>
       </c>
     </row>
@@ -2028,50 +2006,68 @@
       <c r="A28" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" t="n">
-        <v>34</v>
-      </c>
-      <c r="D28" t="n">
-        <v>58</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>338</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
+        <v>338</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>\acs{MPW}-to-methanol with \acs{CC}</t>
+          <t>\acs{MPW}-to-methanol existing</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>\% captured</t>
+          <t>t MPW/h</t>
         </is>
       </c>
     </row>
@@ -2100,10 +2096,10 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>338</v>
+        <v>29</v>
       </c>
       <c r="G29" t="n">
-        <v>338</v>
+        <v>53</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -2130,19 +2126,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="M29" t="n">
+        <v>0</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>\acs{MPW}-to-methanol existing</t>
+          <t>\acs{MPW}-to-methanol existing with \acs{CC}</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>t MPW/h</t>
+          <t>\% captured</t>
         </is>
       </c>
     </row>
@@ -2155,15 +2149,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C30" t="n">
+        <v>106</v>
+      </c>
+      <c r="D30" t="n">
+        <v>157</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2171,49 +2161,41 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>29</v>
+        <v>111</v>
       </c>
       <c r="G30" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I30" t="n">
+        <v>152</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="L30" t="n">
+        <v>139</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>\acs{MPW}-to-methanol existing with \acs{CC}</t>
+          <t>\ce{CO2} electrolysis</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>\% captured</t>
+          <t>t \ce{CO2}/h</t>
         </is>
       </c>
     </row>
@@ -2226,48 +2208,60 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>106</v>
-      </c>
-      <c r="D31" t="n">
-        <v>157</v>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
         <v>111</v>
       </c>
-      <c r="G31" t="n">
-        <v>40</v>
-      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I31" t="n">
-        <v>155</v>
-      </c>
-      <c r="J31" t="n">
-        <v>12</v>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L31" t="n">
-        <v>161</v>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>\ce{CO2} electrolysis</t>
+          <t>\ce{CO2} electrolysis existing</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2280,70 +2274,50 @@
       <c r="A32" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B32" t="n">
+        <v>29</v>
+      </c>
+      <c r="C32" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" t="n">
+        <v>28</v>
+      </c>
+      <c r="E32" t="n">
+        <v>28</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>111</v>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>29</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>28</v>
+      </c>
+      <c r="K32" t="n">
+        <v>28</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>\ce{CO2} electrolysis existing</t>
+          <t>\acs{ASU}</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>t \ce{CO2}/h</t>
+          <t>MW electricity</t>
         </is>
       </c>
     </row>
@@ -2351,45 +2325,61 @@
       <c r="A33" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B33" t="n">
-        <v>29</v>
-      </c>
-      <c r="C33" t="n">
-        <v>10</v>
-      </c>
-      <c r="D33" t="n">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
         <v>28</v>
       </c>
-      <c r="E33" t="n">
+      <c r="G33" t="n">
         <v>28</v>
       </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>29</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
         <v>28</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
       </c>
       <c r="M33" t="n">
         <v>28</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>\acs{ASU}</t>
+          <t>\acs{ASU} existing</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2402,70 +2392,50 @@
       <c r="A34" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B34" t="n">
+        <v>128</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>125</v>
       </c>
       <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" t="n">
         <v>28</v>
       </c>
-      <c r="G34" t="n">
-        <v>28</v>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>334</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>\acs{ASU} existing</t>
+          <t>Gas-fired boiler</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>MW electricity</t>
+          <t>MW gas</t>
         </is>
       </c>
     </row>
@@ -2473,45 +2443,63 @@
       <c r="A35" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="B35" t="n">
-        <v>128</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
         <v>125</v>
       </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
       <c r="G35" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" t="n">
-        <v>2</v>
-      </c>
-      <c r="I35" t="n">
-        <v>27</v>
-      </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>44</v>
-      </c>
-      <c r="L35" t="n">
-        <v>413</v>
+        <v>125</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>334</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Gas-fired boiler</t>
+          <t>Gas-fired boiler existing</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -2524,66 +2512,50 @@
       <c r="A36" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B36" t="n">
+        <v>65</v>
+      </c>
+      <c r="C36" t="n">
+        <v>139</v>
+      </c>
+      <c r="D36" t="n">
+        <v>124</v>
+      </c>
+      <c r="E36" t="n">
+        <v>64</v>
       </c>
       <c r="F36" t="n">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>125</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>51</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>123</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>457</v>
+        <v>425</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Gas-fired boiler existing</t>
+          <t>Electric boiler</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>MW gas</t>
+          <t>MW electricity</t>
         </is>
       </c>
     </row>
@@ -2591,45 +2563,63 @@
       <c r="A37" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="B37" t="n">
-        <v>65</v>
-      </c>
-      <c r="C37" t="n">
-        <v>139</v>
-      </c>
-      <c r="D37" t="n">
-        <v>124</v>
-      </c>
-      <c r="E37" t="n">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
         <v>64</v>
       </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
       <c r="G37" t="n">
-        <v>51</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>84</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>42</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
+        <v>64</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M37" t="n">
-        <v>363</v>
+        <v>1</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Electric boiler</t>
+          <t>Electric boiler existing</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -2642,66 +2632,50 @@
       <c r="A38" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B38" t="n">
+        <v>7225</v>
+      </c>
+      <c r="C38" t="n">
+        <v>5629</v>
+      </c>
+      <c r="D38" t="n">
+        <v>135</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4527</v>
       </c>
       <c r="F38" t="n">
-        <v>64</v>
+        <v>4589</v>
       </c>
       <c r="G38" t="n">
-        <v>64</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>8111</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1395</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4483</v>
       </c>
       <c r="L38" t="n">
-        <v>42</v>
+        <v>4414</v>
       </c>
       <c r="M38" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Electric boiler existing</t>
+          <t>Ammonia tank</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>MW electricity</t>
+          <t>tonne</t>
         </is>
       </c>
     </row>
@@ -2709,45 +2683,61 @@
       <c r="A39" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="B39" t="n">
-        <v>7225</v>
-      </c>
-      <c r="C39" t="n">
-        <v>5629</v>
-      </c>
-      <c r="D39" t="n">
-        <v>135</v>
-      </c>
-      <c r="E39" t="n">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
         <v>4527</v>
       </c>
-      <c r="F39" t="n">
-        <v>4589</v>
-      </c>
       <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>8031</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1396</v>
-      </c>
-      <c r="J39" t="n">
-        <v>76</v>
-      </c>
-      <c r="K39" t="n">
-        <v>29</v>
+        <v>9117</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L39" t="n">
-        <v>1129</v>
+        <v>4483</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>8897</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Ammonia tank</t>
+          <t>Ammonia tank existing</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2760,66 +2750,50 @@
       <c r="A40" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B40" t="n">
+        <v>1212</v>
+      </c>
+      <c r="C40" t="n">
+        <v>5963</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1639</v>
       </c>
       <c r="F40" t="n">
-        <v>4527</v>
+        <v>6414</v>
       </c>
       <c r="G40" t="n">
-        <v>9117</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1337</v>
+      </c>
+      <c r="I40" t="n">
+        <v>4798</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1724</v>
       </c>
       <c r="L40" t="n">
-        <v>29</v>
+        <v>6408</v>
       </c>
       <c r="M40" t="n">
-        <v>1157</v>
+        <v>0</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Ammonia tank existing</t>
+          <t>Li-ion battery</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>tonne</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -2827,45 +2801,61 @@
       <c r="A41" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="B41" t="n">
-        <v>1212</v>
-      </c>
-      <c r="C41" t="n">
-        <v>5963</v>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" t="n">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
         <v>1639</v>
       </c>
-      <c r="F41" t="n">
-        <v>6414</v>
-      </c>
       <c r="G41" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" t="n">
-        <v>1339</v>
-      </c>
-      <c r="I41" t="n">
-        <v>4489</v>
-      </c>
-      <c r="J41" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" t="n">
-        <v>752</v>
+        <v>8053</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L41" t="n">
-        <v>4351</v>
+        <v>1724</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>8133</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Li-ion battery</t>
+          <t>Li-ion battery existing</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -2878,66 +2868,50 @@
       <c r="A42" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>6461</v>
+      </c>
+      <c r="D42" t="n">
+        <v>50</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>1639</v>
+        <v>9813</v>
       </c>
       <c r="G42" t="n">
-        <v>8053</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1056</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>752</v>
+        <v>2110</v>
       </c>
       <c r="M42" t="n">
-        <v>5102</v>
+        <v>0</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Li-ion battery existing</t>
+          <t>\ce{CO2} buffer storage</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>tonne</t>
         </is>
       </c>
     </row>
@@ -2945,45 +2919,65 @@
       <c r="A43" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="n">
-        <v>6461</v>
-      </c>
-      <c r="D43" t="n">
-        <v>50</v>
-      </c>
-      <c r="E43" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" t="n">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
         <v>9813</v>
       </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>41</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
-        <v>7</v>
-      </c>
-      <c r="L43" t="n">
-        <v>4817</v>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M43" t="n">
-        <v>0</v>
+        <v>2110</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>\ce{CO2} buffer storage</t>
+          <t>\ce{CO2} buffer storage existing</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -2996,68 +2990,50 @@
       <c r="A44" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B44" t="n">
+        <v>162</v>
+      </c>
+      <c r="C44" t="n">
+        <v>71</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>166</v>
+      </c>
+      <c r="F44" t="n">
+        <v>8342</v>
       </c>
       <c r="G44" t="n">
-        <v>9813</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>129</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>238</v>
       </c>
       <c r="L44" t="n">
-        <v>7</v>
+        <v>411</v>
       </c>
       <c r="M44" t="n">
-        <v>4824</v>
+        <v>0</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>\ce{CO2} buffer storage existing</t>
+          <t>Hydrogen tank</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>tonne</t>
+          <t>MWh</t>
         </is>
       </c>
     </row>
@@ -3065,45 +3041,61 @@
       <c r="A45" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="B45" t="n">
-        <v>162</v>
-      </c>
-      <c r="C45" t="n">
-        <v>71</v>
-      </c>
-      <c r="D45" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" t="n">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
         <v>166</v>
       </c>
-      <c r="F45" t="n">
-        <v>8342</v>
-      </c>
       <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>125</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
+        <v>8508</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>238</v>
       </c>
       <c r="M45" t="n">
-        <v>0</v>
+        <v>649</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Hydrogen tank</t>
+          <t>Hydrogen tank existing</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3116,70 +3108,50 @@
       <c r="A46" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="n">
+        <v>7112</v>
+      </c>
+      <c r="D46" t="n">
+        <v>49</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>166</v>
+        <v>1365</v>
       </c>
       <c r="G46" t="n">
-        <v>8508</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>3307</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>9</v>
+      </c>
+      <c r="L46" t="n">
+        <v>497</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Hydrogen tank existing</t>
+          <t>Ethylene tank</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>tonne</t>
         </is>
       </c>
     </row>
@@ -3187,45 +3159,63 @@
       <c r="A47" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="B47" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" t="n">
-        <v>7112</v>
-      </c>
-      <c r="D47" t="n">
-        <v>49</v>
-      </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="n">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
         <v>1365</v>
       </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>500</v>
-      </c>
-      <c r="J47" t="n">
-        <v>80</v>
-      </c>
-      <c r="K47" t="n">
-        <v>7</v>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L47" t="n">
-        <v>500</v>
+        <v>9</v>
       </c>
       <c r="M47" t="n">
-        <v>0</v>
+        <v>506</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Ethylene tank</t>
+          <t>Ethylene tank existing</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -3238,63 +3228,45 @@
       <c r="A48" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" t="n">
+        <v>571</v>
+      </c>
+      <c r="D48" t="n">
+        <v>20</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>4449</v>
       </c>
       <c r="G48" t="n">
-        <v>1365</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>5691</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>9</v>
       </c>
       <c r="L48" t="n">
-        <v>7</v>
+        <v>9219</v>
       </c>
       <c r="M48" t="n">
-        <v>507</v>
+        <v>0</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Ethylene tank existing</t>
+          <t>Propylene tank</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -3307,117 +3279,66 @@
       <c r="A49" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="B49" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" t="n">
-        <v>571</v>
-      </c>
-      <c r="D49" t="n">
-        <v>20</v>
-      </c>
-      <c r="E49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" t="n">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
         <v>4449</v>
       </c>
-      <c r="G49" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" t="n">
-        <v>8736</v>
-      </c>
-      <c r="J49" t="n">
-        <v>131</v>
-      </c>
-      <c r="K49" t="n">
-        <v>6</v>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L49" t="n">
-        <v>9252</v>
+        <v>9</v>
       </c>
       <c r="M49" t="n">
-        <v>0</v>
+        <v>9227</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Propylene tank</t>
+          <t>Propylene tank existing</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
-        <is>
-          <t>tonne</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>4449</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L50" t="n">
-        <v>6</v>
-      </c>
-      <c r="M50" t="n">
-        <v>9257</v>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>Propylene tank existing</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
         <is>
           <t>tonne</t>
         </is>

</xml_diff>